<commit_message>
The Furever Home - Bay Area Pet Adoption Website
</commit_message>
<xml_diff>
--- a/Website Spec template.xlsx
+++ b/Website Spec template.xlsx
@@ -8,20 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Pet Proj 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93DEA05-7975-43F1-AE65-B3D1423AE538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F969D80E-F907-4E9C-A951-8C8DD09B7836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Website Technical Specification" sheetId="1" r:id="rId1"/>
     <sheet name="Issue fix" sheetId="6" r:id="rId2"/>
-    <sheet name="To do" sheetId="7" r:id="rId3"/>
-    <sheet name="prompt" sheetId="5" r:id="rId4"/>
-    <sheet name="objective" sheetId="3" r:id="rId5"/>
+    <sheet name="prompt" sheetId="5" r:id="rId3"/>
+    <sheet name="objective" sheetId="3" r:id="rId4"/>
   </sheets>
   <externalReferences>
+    <externalReference r:id="rId5"/>
     <externalReference r:id="rId6"/>
-    <externalReference r:id="rId7"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Website Technical Specification'!$B$1:$E$46</definedName>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="108">
   <si>
     <t>PROJECT NAME</t>
   </si>
@@ -78,12 +77,6 @@
     <t>WEBSITE FUNCTIONAL REQUIREMENTS TEMPLATE</t>
   </si>
   <si>
-    <t xml:space="preserve">It can be useful to remind internal users what your purpose is and is essential to good function and design to explain this to external vendors. What does your organization do? When was your organization founded and why? Size of company and location. Main products and services. </t>
-  </si>
-  <si>
-    <t>who are u</t>
-  </si>
-  <si>
     <t>website needed because</t>
   </si>
   <si>
@@ -235,9 +228,6 @@
   </si>
   <si>
     <t>AWS S3 bucket free hosting</t>
-  </si>
-  <si>
-    <t>Nightly refresh and update the availble pets on my website based on if other shelers have new or removed pet.</t>
   </si>
   <si>
     <t>nightly batch/ crone job</t>
@@ -250,21 +240,6 @@
     <t>Issue and how to fix</t>
   </si>
   <si>
-    <t>Filters are not sorting pet based on the filed in category. Ex. Only dogs should be visible if I select dog in filter</t>
-  </si>
-  <si>
-    <t>Not able to open detailed info about pet after clicking the pet image</t>
-  </si>
-  <si>
-    <t>Make menu or submenu fit into a single line</t>
-  </si>
-  <si>
-    <t>Make the roadmap fit into a single line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pet match quiz should be collapsable. It should show question and options only when u click on it. </t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -277,36 +252,6 @@
     <t>Wishlist</t>
   </si>
   <si>
-    <t>Pending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apply filter button, should refresh pets and show best matches on tops. Rt now I see both dogs and cats when I click cats. </t>
-  </si>
-  <si>
-    <t>Entire</t>
-  </si>
-  <si>
-    <t>Add footer to website with some info of site, links to tabs on our site, partner shelter and disclaimer that pets may change and contact indiv. Shelters.</t>
-  </si>
-  <si>
-    <t>Pet info should open in full screen</t>
-  </si>
-  <si>
-    <t>Example pic:</t>
-  </si>
-  <si>
-    <t>Filters on left side of page and pets on right</t>
-  </si>
-  <si>
-    <t>Logo: cute dog and cat</t>
-  </si>
-  <si>
-    <t>Color theme: Main Text: Dark Charcoal. Background: Warm Cream .Buttons/Links: Bright Teal .Dusty Pink Use this for borders, icons, and faded backgrounds.</t>
-  </si>
-  <si>
-    <t>New tab</t>
-  </si>
-  <si>
     <t>Vission, misssion, values</t>
   </si>
   <si>
@@ -361,13 +306,64 @@
     <t>Checklist</t>
   </si>
   <si>
-    <t>Sort tabs on top pof the page as table is on the right</t>
-  </si>
-  <si>
-    <t>use logo</t>
-  </si>
-  <si>
-    <t>in scrolling frame, use diff images like event, adoption, stories, mission</t>
+    <t>New version updates to stand out:</t>
+  </si>
+  <si>
+    <t>done</t>
+  </si>
+  <si>
+    <t>to do</t>
+  </si>
+  <si>
+    <t>hmm</t>
+  </si>
+  <si>
+    <t>Donations tab</t>
+  </si>
+  <si>
+    <t># pets adopted</t>
+  </si>
+  <si>
+    <t>All Pets- live feed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home </t>
+  </si>
+  <si>
+    <t># of downloads</t>
+  </si>
+  <si>
+    <t>Google sheet database</t>
+  </si>
+  <si>
+    <t>Entire website</t>
+  </si>
+  <si>
+    <t>Nightly refresh and update the availble pets on my website based on if other shelters have new or removed pet.</t>
+  </si>
+  <si>
+    <t>Partner shelters</t>
+  </si>
+  <si>
+    <t>Phase 2</t>
+  </si>
+  <si>
+    <t>Interest form below pet finder</t>
+  </si>
+  <si>
+    <t>Sign In/ up</t>
+  </si>
+  <si>
+    <t>Add new contact info</t>
+  </si>
+  <si>
+    <t>roadmap with pics</t>
+  </si>
+  <si>
+    <t>Banner take to the petfnder</t>
+  </si>
+  <si>
+    <t>I like the website/app button: RIGHT ALIGN MOVE</t>
   </si>
 </sst>
 </file>
@@ -507,7 +503,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -568,6 +564,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="17">
     <border>
@@ -909,64 +911,64 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1007,23 +1009,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>598649</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>258917</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>77020</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>295276</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>101327</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0EEE4DD-2D2A-FAE2-FFDD-7C88ECE13CCB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DFA54099-6EF2-7E95-DCBB-36FA9C5FBEA3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1039,8 +1041,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1666875" y="3400425"/>
-          <a:ext cx="12479492" cy="5877745"/>
+          <a:off x="15171899" y="2724150"/>
+          <a:ext cx="5868827" cy="2777852"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1051,23 +1053,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>847725</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>277969</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>115126</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>200656</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>162457</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DFA54099-6EF2-7E95-DCBB-36FA9C5FBEA3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9ADC865C-15AB-7EAD-891C-9FF26DFBA7EF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1083,8 +1085,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1666875" y="9401175"/>
-          <a:ext cx="12498544" cy="5915851"/>
+          <a:off x="9258300" y="2952750"/>
+          <a:ext cx="4525006" cy="3810532"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1412,32 +1414,32 @@
       <c r="E1" s="6"/>
     </row>
     <row r="2" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="44"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="47"/>
     </row>
     <row r="3" spans="2:5" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
+      <c r="C3" s="48" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="49"/>
+      <c r="E3" s="50"/>
     </row>
     <row r="4" spans="2:5" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E4" s="12"/>
     </row>
@@ -1448,22 +1450,22 @@
       <c r="E5" s="14"/>
     </row>
     <row r="6" spans="2:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
     </row>
     <row r="7" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E7" s="6"/>
     </row>
@@ -1472,10 +1474,10 @@
         <v>1</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E8" s="6"/>
     </row>
@@ -1484,10 +1486,10 @@
         <v>1</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E9" s="6"/>
     </row>
@@ -1496,10 +1498,10 @@
         <v>1</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E10" s="6"/>
     </row>
@@ -1508,10 +1510,10 @@
         <v>2</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E11" s="6"/>
     </row>
@@ -1520,10 +1522,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E12" s="6"/>
     </row>
@@ -1532,10 +1534,10 @@
         <v>2</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E13" s="6"/>
     </row>
@@ -1544,10 +1546,10 @@
         <v>2</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E14" s="6"/>
     </row>
@@ -1556,10 +1558,10 @@
         <v>1</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E15" s="6"/>
     </row>
@@ -1568,10 +1570,10 @@
         <v>1</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E16" s="6"/>
     </row>
@@ -1580,10 +1582,10 @@
         <v>1</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E17" s="6"/>
     </row>
@@ -1592,10 +1594,10 @@
         <v>2</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>65</v>
+        <v>99</v>
       </c>
       <c r="E18" s="6"/>
     </row>
@@ -1614,12 +1616,12 @@
     </row>
     <row r="21" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="36"/>
+      <c r="D21" s="42"/>
       <c r="E21" s="1" t="s">
         <v>7</v>
       </c>
@@ -1628,62 +1630,62 @@
       <c r="B22" s="22">
         <v>1</v>
       </c>
-      <c r="C22" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" s="39"/>
+      <c r="C22" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" s="40"/>
       <c r="E22" s="25" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="22"/>
-      <c r="C23" s="38" t="s">
-        <v>45</v>
-      </c>
-      <c r="D23" s="39"/>
+      <c r="C23" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="40"/>
       <c r="E23" s="25" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="22"/>
-      <c r="C24" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="D24" s="39"/>
+      <c r="C24" s="39" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" s="40"/>
       <c r="E24" s="25" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="22.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="22"/>
       <c r="C25" s="23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D25" s="24"/>
       <c r="E25" s="25" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="22"/>
       <c r="C26" s="22" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D26" s="24"/>
       <c r="E26" s="25" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="2:5" ht="8.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="26"/>
-      <c r="C27" s="40" t="s">
-        <v>56</v>
-      </c>
-      <c r="D27" s="41"/>
+      <c r="C27" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="44"/>
       <c r="E27" s="27" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1710,42 +1712,42 @@
       <c r="B31" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C31" s="35" t="s">
+      <c r="C31" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="D31" s="36"/>
+      <c r="D31" s="42"/>
       <c r="E31" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="32" spans="2:5" s="16" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="22"/>
-      <c r="C32" s="38"/>
-      <c r="D32" s="39"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="40"/>
       <c r="E32" s="25"/>
     </row>
     <row r="33" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="22"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="39"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="40"/>
       <c r="E33" s="25"/>
     </row>
     <row r="34" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="22"/>
-      <c r="C34" s="38"/>
-      <c r="D34" s="39"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="40"/>
       <c r="E34" s="25"/>
     </row>
     <row r="35" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="22"/>
-      <c r="C35" s="38"/>
-      <c r="D35" s="39"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="40"/>
       <c r="E35" s="25"/>
     </row>
     <row r="36" spans="2:5" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="26"/>
-      <c r="C36" s="40"/>
-      <c r="D36" s="41"/>
+      <c r="C36" s="43"/>
+      <c r="D36" s="44"/>
       <c r="E36" s="27"/>
     </row>
     <row r="37" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1764,12 +1766,12 @@
     </row>
     <row r="39" spans="2:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C39" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="D39" s="36"/>
+      <c r="D39" s="42"/>
       <c r="E39" s="1" t="s">
         <v>7</v>
       </c>
@@ -1778,22 +1780,22 @@
       <c r="B40" s="22">
         <v>1</v>
       </c>
-      <c r="C40" s="38" t="s">
-        <v>27</v>
-      </c>
-      <c r="D40" s="39"/>
+      <c r="C40" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D40" s="40"/>
       <c r="E40" s="25" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41" spans="2:5" s="16" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="22"/>
-      <c r="C41" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="D41" s="39"/>
+      <c r="C41" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="D41" s="40"/>
       <c r="E41" s="25" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="42" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1814,20 +1816,20 @@
       <c r="B44" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C44" s="35" t="s">
+      <c r="C44" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="D44" s="36"/>
+      <c r="D44" s="42"/>
       <c r="E44" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="45" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="22"/>
-      <c r="C45" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="D45" s="39"/>
+      <c r="C45" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="D45" s="40"/>
       <c r="E45" s="25"/>
     </row>
     <row r="46" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1888,11 +1890,6 @@
     <row r="81" ht="100.35" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C41:D41"/>
     <mergeCell ref="C33:D33"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="C35:D35"/>
@@ -1907,6 +1904,11 @@
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C41:D41"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -1921,12 +1923,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43A120F6-F432-4C36-B549-797F86B2FDBD}">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" style="31" customWidth="1"/>
-    <col min="2" max="2" width="14.875" style="31" customWidth="1"/>
-    <col min="3" max="3" width="56.5" style="31" customWidth="1"/>
+    <col min="2" max="2" width="19.875" style="31" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="88.5" style="31" customWidth="1"/>
     <col min="4" max="6" width="9" style="31"/>
     <col min="7" max="7" width="11.375" style="31" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.75" style="31" customWidth="1"/>
@@ -1937,122 +1939,122 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="32" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="33" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D1" s="32" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="E1" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
+        <v>67</v>
+      </c>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="30">
         <v>1</v>
       </c>
       <c r="B2" s="30" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2" s="34" t="s">
-        <v>70</v>
+        <v>107</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="E2" s="49">
-        <v>46188</v>
-      </c>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
+        <v>68</v>
+      </c>
+      <c r="E2" s="36">
+        <v>46197</v>
+      </c>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="30">
         <v>2</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>50</v>
+        <v>94</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="D3" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="49">
-        <v>46188</v>
-      </c>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
+        <v>68</v>
+      </c>
+      <c r="E3" s="36">
+        <v>46197</v>
+      </c>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="30">
         <v>3</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>49</v>
+        <v>98</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>69</v>
+        <v>103</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="E4" s="49">
-        <v>46188</v>
-      </c>
-      <c r="F4" s="51"/>
-      <c r="G4" s="51"/>
+        <v>68</v>
+      </c>
+      <c r="E4" s="36">
+        <v>46197</v>
+      </c>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="30">
         <v>4</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>53</v>
+        <v>100</v>
       </c>
       <c r="C5" s="34" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="E5" s="49">
-        <v>46188</v>
-      </c>
-      <c r="F5" s="51"/>
-      <c r="G5" s="51"/>
+        <v>68</v>
+      </c>
+      <c r="E5" s="36">
+        <v>46197</v>
+      </c>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="30">
         <v>5</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>71</v>
+        <v>105</v>
       </c>
       <c r="D6" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="36">
+        <v>46197</v>
+      </c>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="K6" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="L6" s="37" t="s">
         <v>76</v>
-      </c>
-      <c r="E6" s="49">
-        <v>46188</v>
-      </c>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="K6" s="50" t="s">
-        <v>102</v>
-      </c>
-      <c r="L6" s="50" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -2060,35 +2062,35 @@
         <v>6</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C7" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="E7" s="36">
+        <v>46197</v>
+      </c>
+      <c r="F7" s="38"/>
+      <c r="G7" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="D7" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="49">
-        <v>46188</v>
-      </c>
-      <c r="F7" s="51"/>
-      <c r="G7" s="48" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" s="48" t="s">
-        <v>91</v>
-      </c>
-      <c r="I7" s="48" t="s">
-        <v>95</v>
-      </c>
-      <c r="J7" s="48" t="s">
-        <v>92</v>
-      </c>
-      <c r="K7" s="48" t="s">
-        <v>103</v>
-      </c>
-      <c r="L7" s="48" t="s">
+      <c r="H7" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="I7" s="35" t="s">
         <v>77</v>
+      </c>
+      <c r="J7" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="K7" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="L7" s="54" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -2096,26 +2098,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>53</v>
+        <v>95</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="D8" s="30" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="E8" s="30"/>
-      <c r="F8" s="52"/>
       <c r="G8" s="30" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="H8" s="30"/>
       <c r="I8" s="30" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="J8" s="30"/>
       <c r="K8" s="30" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="L8" s="30"/>
     </row>
@@ -2124,26 +2125,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="E9" s="30"/>
+      <c r="G9" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="H9" s="30"/>
+      <c r="I9" s="52" t="s">
         <v>80</v>
-      </c>
-      <c r="C9" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="D9" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="E9" s="30"/>
-      <c r="F9" s="52"/>
-      <c r="G9" s="30" t="s">
-        <v>100</v>
-      </c>
-      <c r="H9" s="30"/>
-      <c r="I9" s="53" t="s">
-        <v>98</v>
       </c>
       <c r="J9" s="30"/>
       <c r="K9" s="30" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="L9" s="30"/>
     </row>
@@ -2152,22 +2152,21 @@
         <v>9</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D10" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="E10" s="30"/>
+      <c r="G10" s="30" t="s">
         <v>78</v>
-      </c>
-      <c r="E10" s="30"/>
-      <c r="F10" s="52"/>
-      <c r="G10" s="30" t="s">
-        <v>96</v>
       </c>
       <c r="H10" s="30"/>
       <c r="I10" s="30" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="J10" s="30"/>
       <c r="K10" s="30"/>
@@ -2177,23 +2176,16 @@
       <c r="A11" s="30">
         <v>10</v>
       </c>
-      <c r="B11" s="30" t="s">
-        <v>80</v>
-      </c>
-      <c r="C11" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="D11" s="30" t="s">
-        <v>78</v>
-      </c>
+      <c r="B11" s="30"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="30"/>
       <c r="E11" s="30"/>
-      <c r="F11" s="52"/>
       <c r="G11" s="30" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="H11" s="30"/>
-      <c r="I11" s="53" t="s">
-        <v>101</v>
+      <c r="I11" s="30" t="s">
+        <v>83</v>
       </c>
       <c r="J11" s="30"/>
       <c r="K11" s="30"/>
@@ -2203,20 +2195,14 @@
       <c r="A12" s="30">
         <v>11</v>
       </c>
-      <c r="B12" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>82</v>
-      </c>
-      <c r="D12" s="30" t="s">
-        <v>78</v>
-      </c>
+      <c r="B12" s="30"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="30"/>
       <c r="E12" s="30"/>
       <c r="G12" s="30"/>
       <c r="H12" s="30"/>
       <c r="I12" s="30" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="J12" s="30"/>
       <c r="K12" s="30"/>
@@ -2226,35 +2212,48 @@
       <c r="A13" s="30">
         <v>12</v>
       </c>
-      <c r="B13" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" s="34" t="s">
-        <v>106</v>
-      </c>
-      <c r="D13" s="30" t="s">
-        <v>78</v>
-      </c>
+      <c r="B13" s="30"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="30"/>
       <c r="E13" s="30"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="30">
         <v>13</v>
       </c>
-      <c r="B14" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="34" t="s">
-        <v>84</v>
-      </c>
-      <c r="D14" s="30" t="s">
-        <v>78</v>
-      </c>
+      <c r="B14" s="30"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="30"/>
       <c r="E14" s="30"/>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C17" s="31" t="s">
-        <v>83</v>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F16" s="31" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G19" s="31" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="23" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G23" s="31" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G26" s="31" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="29" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G29" s="53" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G31" s="31" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -2264,26 +2263,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64CE4FFD-E3F2-4B32-8443-D96A7827FEC8}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFBCDCB-D827-4011-A151-483F8A3979A8}">
   <dimension ref="B2"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -2293,7 +2272,7 @@
   <sheetData>
     <row r="2" spans="2:2" ht="173.25" x14ac:dyDescent="0.25">
       <c r="B2" s="29" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2301,9 +2280,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C861D98-A3D4-48B1-98A0-8E00BCA30AEA}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.125" customWidth="1"/>
@@ -2316,10 +2295,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
         <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2340,26 +2319,18 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
         <v>18</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
         <v>21</v>
-      </c>
-      <c r="B11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>